<commit_message>
No significant changes. Start of 2026-Q2
</commit_message>
<xml_diff>
--- a/Admin/Opening and Closing Price Cheat Table.xlsx
+++ b/Admin/Opening and Closing Price Cheat Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading_Algo/Admin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{23DDF59B-E8BC-405C-8550-BE27D8A4AF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECB41062-046F-469A-A745-806B84376FDB}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="8_{23DDF59B-E8BC-405C-8550-BE27D8A4AF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C52FC0FB-C8AD-443C-9853-04D7A23C65C0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8D7F9898-85BA-4D87-B10C-1CA563D32779}"/>
   </bookViews>
@@ -121,7 +121,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -146,6 +146,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -200,14 +218,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -218,6 +230,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -233,6 +255,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -564,286 +590,286 @@
   </cols>
   <sheetData>
     <row r="6" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K6" s="1" t="s">
+      <c r="K6" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="3" t="s">
+      <c r="L6" s="12"/>
+      <c r="M6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="N6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="O6" s="3" t="s">
+      <c r="O6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P6" s="3" t="s">
+      <c r="P6" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="Q6" s="3" t="s">
+      <c r="Q6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="R6" s="3" t="s">
+      <c r="R6" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K7" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="N7" s="6" t="s">
+      <c r="K7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="N7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="O7" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="P7" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q7" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="R7" s="6" t="s">
+      <c r="O7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="P7" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="R7" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K8" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="N8" s="6" t="s">
+      <c r="K8" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="O8" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="P8" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q8" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="R8" s="6" t="s">
+      <c r="O8" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="P8" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="R8" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K9" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="N9" s="9" t="s">
+      <c r="K9" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="N9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="O9" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="P9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="R9" s="9" t="s">
+      <c r="O9" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P9" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="R9" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K10" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="M10" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="N10" s="9" t="s">
+      <c r="K10" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N10" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="O10" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="P10" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q10" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="R10" s="9" t="s">
+      <c r="O10" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P10" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="R10" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K11" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="L11" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="M11" s="6" t="s">
+      <c r="K11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="6" t="s">
+      <c r="N11" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="O11" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="s">
+      <c r="O11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="P11" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="Q11" s="6" t="s">
+      <c r="Q11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="R11" s="6" t="s">
+      <c r="R11" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K12" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="L12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="N12" s="6" t="s">
+      <c r="K12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="N12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="O12" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="P12" s="6" t="s">
+      <c r="O12" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="P12" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="Q12" s="6" t="s">
+      <c r="Q12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="R12" s="6" t="s">
+      <c r="R12" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K13" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="M13" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="N13" s="9" t="s">
+      <c r="K13" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="N13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="O13" s="9" t="s">
+      <c r="O13" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="P13" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="R13" s="9" t="s">
+      <c r="P13" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="R13" s="7" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K14" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="M14" s="12" t="s">
+      <c r="K14" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="M14" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="N14" s="12" t="s">
+      <c r="N14" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="O14" s="12" t="s">
+      <c r="O14" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="P14" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="R14" s="12" t="s">
+      <c r="P14" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="R14" s="10" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="15" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K15" s="4" t="s">
+      <c r="K15" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="L15" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="N15" s="6" t="s">
+      <c r="L15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N15" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="O15" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="P15" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q15" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="R15" s="6" t="s">
+      <c r="O15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P15" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="R15" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="16" spans="11:18" x14ac:dyDescent="0.25">
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="L16" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="N16" s="6" t="s">
+      <c r="L16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N16" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="O16" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="P16" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q16" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="R16" s="6" t="s">
+      <c r="O16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P16" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="R16" s="4" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>